<commit_message>
fix(deliverables): direct links, Ozvor branding, kit fallback
</commit_message>
<xml_diff>
--- a/apps/web/public/downloads/LLM-Citation-Tracker.xlsx
+++ b/apps/web/public/downloads/LLM-Citation-Tracker.xlsx
@@ -807,14 +807,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LLM Citation Tracker — by TrustIndex AI</t>
+          <t>LLM Citation Tracker — by Ozvor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>trustindexai.com · hello@trustindexai.com</t>
+          <t>ozvor.com · hello@ozvor.com</t>
         </is>
       </c>
     </row>
@@ -984,14 +984,14 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>When 10 queries isn't enough coverage, start free at trustindexai.com. TrustIndex AI monitors all five engines automatically, scores your AI visibility (TrustIndex Score), benchmarks competitors, and tells you what to publish next. Growth plan $99/mo (or $831/yr founder pricing).</t>
+          <t>When 10 queries isn't enough coverage, start free at ozvor.com. Ozvor monitors all five engines automatically, scores your AI visibility (Ozvor AI Visibility Score), benchmarks competitors, and tells you what to publish next. Growth plan $99/mo (or $831/yr founder pricing).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Outgrown the spreadsheet? TrustIndex AI — the AI Search Trust Intelligence platform for SMBs. Start free at trustindexai.com · hello@trustindexai.com.</t>
+          <t>Outgrown the spreadsheet? Ozvor — the AI Search Trust Intelligence platform for SMBs. Start free at ozvor.com · hello@ozvor.com.</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Outgrown the spreadsheet? TrustIndex AI monitors all 5 engines automatically, scores your AI visibility, and benchmarks competitors. Start free at trustindexai.com.</t>
+          <t>Outgrown the spreadsheet? Ozvor monitors all 5 engines automatically, scores your AI visibility, and benchmarks competitors. Start free at ozvor.com.</t>
         </is>
       </c>
     </row>

</xml_diff>